<commit_message>
Refine header nav + booking widget, add table block
- Restyle booking widget to the navy inline look (tab icons, underline
  fields, gold circular search) and inject it site-wide, not just the homepage.
- Fix mega-menu hover: add a close delay so the pointer can reach the panel;
  remove the dropdown caret pseudo-elements under Plan/Fly/Explore/Help.
- Add a table block + parser so the baggage-allowance data table renders as a
  real striped table instead of a broken "flights" block.
- Extend the cleanup transformer to strip stray source chrome (off-canvas
  menu, date-range pickers, Salesforce live-chat button) and re-import content.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -40,7 +40,7 @@
     <t>baggage-allowance.report.json</t>
   </si>
   <si>
-    <t>["accordion-faq","accordion-faq"]</t>
+    <t>["accordion-faq","accordion-faq","table"]</t>
   </si>
   <si>
     <t>baggage-allowance</t>
@@ -52,7 +52,7 @@
     <t>content-page</t>
   </si>
   <si>
-    <t>2026-07-14T13:20:57.669Z</t>
+    <t>2026-07-19T09:48:26.006Z</t>
   </si>
   <si>
     <t>Nile Air – Your Journey, Our Care</t>
@@ -73,7 +73,7 @@
     <t>home-landing</t>
   </si>
   <si>
-    <t>2026-07-14T13:20:21.042Z</t>
+    <t>2026-07-19T09:47:55.705Z</t>
   </si>
   <si>
     <t>https://www.nileair.com/</t>
@@ -88,7 +88,7 @@
     <t>nileair-holidays</t>
   </si>
   <si>
-    <t>2026-07-14T13:21:09.399Z</t>
+    <t>2026-07-19T09:48:39.465Z</t>
   </si>
   <si>
     <t>https://www.nileair.com/nileair-holidays</t>
@@ -103,7 +103,7 @@
     <t>travelling-pets</t>
   </si>
   <si>
-    <t>2026-07-14T13:20:48.067Z</t>
+    <t>2026-07-19T09:48:13.626Z</t>
   </si>
   <si>
     <t>https://www.nileair.com/travelling-pets</t>

</xml_diff>